<commit_message>
ajout des prix par grade pour le catalogue de la cote d'ivoire 2.1
</commit_message>
<xml_diff>
--- a/PRIX CIV 2.xlsx
+++ b/PRIX CIV 2.xlsx
@@ -888,19 +888,19 @@
         <v>14</v>
       </c>
       <c r="B2" s="1">
-        <v>14782</v>
+        <v>14682</v>
       </c>
       <c r="C2" s="1">
-        <v>10916</v>
+        <v>10816</v>
       </c>
       <c r="D2" s="1">
-        <v>9680</v>
+        <v>9580</v>
       </c>
       <c r="E2" s="1">
-        <v>8906</v>
+        <v>8806</v>
       </c>
       <c r="F2" s="1">
-        <v>8134</v>
+        <v>8034</v>
       </c>
       <c r="G2" s="3">
         <v>7.1999999999999995E-2</v>
@@ -911,19 +911,19 @@
         <v>815</v>
       </c>
       <c r="B3" s="1">
-        <v>20484</v>
+        <v>20384</v>
       </c>
       <c r="C3" s="1">
-        <v>15110</v>
+        <v>15009.25</v>
       </c>
       <c r="D3" s="1">
-        <v>13393</v>
+        <v>13293</v>
       </c>
       <c r="E3" s="1">
-        <v>12320</v>
+        <v>12220</v>
       </c>
       <c r="F3" s="1">
-        <v>11247</v>
+        <v>11147</v>
       </c>
       <c r="G3" s="3">
         <v>0.1</v>
@@ -934,7 +934,7 @@
         <v>22</v>
       </c>
       <c r="B4" s="1">
-        <v>29855</v>
+        <v>29755</v>
       </c>
       <c r="C4" s="1">
         <v>2094</v>
@@ -957,19 +957,19 @@
         <v>26</v>
       </c>
       <c r="B5" s="1">
-        <v>12329</v>
+        <v>12229</v>
       </c>
       <c r="C5" s="1">
-        <v>9103</v>
+        <v>9003</v>
       </c>
       <c r="D5" s="1">
-        <v>8073</v>
+        <v>7973</v>
       </c>
       <c r="E5" s="1">
-        <v>7429</v>
+        <v>7329</v>
       </c>
       <c r="F5" s="1">
-        <v>6784</v>
+        <v>6684</v>
       </c>
       <c r="G5" s="3">
         <v>0.06</v>
@@ -980,19 +980,19 @@
         <v>27</v>
       </c>
       <c r="B6" s="1">
-        <v>26602</v>
+        <v>26502</v>
       </c>
       <c r="C6" s="1">
-        <v>19614</v>
+        <v>19514</v>
       </c>
       <c r="D6" s="1">
-        <v>17383</v>
+        <v>17283</v>
       </c>
       <c r="E6" s="1">
-        <v>15988</v>
+        <v>15888</v>
       </c>
       <c r="F6" s="1">
-        <v>14592</v>
+        <v>14492</v>
       </c>
       <c r="G6" s="3">
         <v>0.13</v>
@@ -1003,7 +1003,7 @@
         <v>28</v>
       </c>
       <c r="B7" s="1">
-        <v>6419</v>
+        <v>6319</v>
       </c>
       <c r="C7" s="1">
         <v>4654</v>
@@ -1026,19 +1026,19 @@
         <v>834</v>
       </c>
       <c r="B8" s="1">
-        <v>20484</v>
+        <v>20384</v>
       </c>
       <c r="C8" s="1">
-        <v>15110</v>
+        <v>15010</v>
       </c>
       <c r="D8" s="1">
-        <v>13393</v>
+        <v>13293</v>
       </c>
       <c r="E8" s="1">
-        <v>12320</v>
+        <v>12220</v>
       </c>
       <c r="F8" s="1">
-        <v>11247</v>
+        <v>11147</v>
       </c>
       <c r="G8" s="3">
         <v>0.1</v>
@@ -1049,19 +1049,19 @@
         <v>36</v>
       </c>
       <c r="B9" s="1">
-        <v>26602</v>
+        <v>26502</v>
       </c>
       <c r="C9" s="1">
-        <v>19614</v>
+        <v>19514</v>
       </c>
       <c r="D9" s="1">
-        <v>17383</v>
+        <v>17283</v>
       </c>
       <c r="E9" s="1">
-        <v>15988</v>
+        <v>15888</v>
       </c>
       <c r="F9" s="1">
-        <v>14592</v>
+        <v>14492</v>
       </c>
       <c r="G9" s="3">
         <v>0.13</v>
@@ -1072,19 +1072,19 @@
         <v>37</v>
       </c>
       <c r="B10" s="1">
-        <v>14782</v>
+        <v>14682</v>
       </c>
       <c r="C10" s="1">
-        <v>10916</v>
+        <v>10816</v>
       </c>
       <c r="D10" s="1">
-        <v>9680</v>
+        <v>9580</v>
       </c>
       <c r="E10" s="1">
-        <v>8906</v>
+        <v>8806</v>
       </c>
       <c r="F10" s="1">
-        <v>8134</v>
+        <v>8034</v>
       </c>
       <c r="G10" s="3">
         <v>7.1999999999999995E-2</v>
@@ -1095,19 +1095,19 @@
         <v>40</v>
       </c>
       <c r="B11" s="1">
-        <v>16209</v>
+        <v>16109</v>
       </c>
       <c r="C11" s="1">
-        <v>11958</v>
+        <v>11858</v>
       </c>
       <c r="D11" s="1">
-        <v>10601</v>
+        <v>10501</v>
       </c>
       <c r="E11" s="1">
-        <v>9753</v>
+        <v>9653</v>
       </c>
       <c r="F11" s="1">
-        <v>8905</v>
+        <v>8805</v>
       </c>
       <c r="G11" s="3">
         <v>7.9000000000000001E-2</v>
@@ -1118,19 +1118,19 @@
         <v>48</v>
       </c>
       <c r="B12" s="1">
-        <v>14172</v>
+        <v>14072</v>
       </c>
       <c r="C12" s="1">
-        <v>10455</v>
+        <v>10355</v>
       </c>
       <c r="D12" s="1">
-        <v>9270</v>
+        <v>9170</v>
       </c>
       <c r="E12" s="1">
-        <v>8529</v>
+        <v>8429</v>
       </c>
       <c r="F12" s="1">
-        <v>7789</v>
+        <v>7689</v>
       </c>
       <c r="G12" s="3">
         <v>6.9000000000000006E-2</v>
@@ -1141,19 +1141,19 @@
         <v>51</v>
       </c>
       <c r="B13" s="1">
-        <v>15801</v>
+        <v>15701</v>
       </c>
       <c r="C13" s="1">
-        <v>11659</v>
+        <v>11559</v>
       </c>
       <c r="D13" s="1">
-        <v>10336</v>
+        <v>10236</v>
       </c>
       <c r="E13" s="1">
-        <v>9510</v>
+        <v>9410</v>
       </c>
       <c r="F13" s="1">
-        <v>8684</v>
+        <v>8584</v>
       </c>
       <c r="G13" s="3">
         <v>7.6999999999999999E-2</v>
@@ -1164,19 +1164,19 @@
         <v>61</v>
       </c>
       <c r="B14" s="1">
-        <v>12128</v>
+        <v>12028</v>
       </c>
       <c r="C14" s="1">
-        <v>8954</v>
+        <v>8854</v>
       </c>
       <c r="D14" s="1">
-        <v>7941</v>
+        <v>7841</v>
       </c>
       <c r="E14" s="1">
-        <v>7308</v>
+        <v>7208</v>
       </c>
       <c r="F14" s="1">
-        <v>6672</v>
+        <v>6572</v>
       </c>
       <c r="G14" s="3">
         <v>5.8999999999999997E-2</v>
@@ -1187,19 +1187,19 @@
         <v>63</v>
       </c>
       <c r="B15" s="1">
-        <v>12128</v>
+        <v>12028</v>
       </c>
       <c r="C15" s="1">
-        <v>8954</v>
+        <v>8854</v>
       </c>
       <c r="D15" s="1">
-        <v>7941</v>
+        <v>7841</v>
       </c>
       <c r="E15" s="1">
-        <v>7308</v>
+        <v>7208</v>
       </c>
       <c r="F15" s="1">
-        <v>6672</v>
+        <v>6572</v>
       </c>
       <c r="G15" s="3">
         <v>5.8999999999999997E-2</v>
@@ -1210,19 +1210,19 @@
         <v>64</v>
       </c>
       <c r="B16" s="1">
-        <v>19128</v>
+        <v>19028</v>
       </c>
       <c r="C16" s="1">
-        <v>8954</v>
+        <v>8854</v>
       </c>
       <c r="D16" s="1">
-        <v>7941</v>
+        <v>7841</v>
       </c>
       <c r="E16" s="1">
-        <v>7308</v>
+        <v>7208</v>
       </c>
       <c r="F16" s="1">
-        <v>6672</v>
+        <v>6572</v>
       </c>
       <c r="G16" s="3">
         <v>5.8999999999999997E-2</v>
@@ -1233,19 +1233,19 @@
         <v>65</v>
       </c>
       <c r="B17" s="1">
-        <v>14775</v>
+        <v>14675</v>
       </c>
       <c r="C17" s="1">
-        <v>10916</v>
+        <v>10816</v>
       </c>
       <c r="D17" s="1">
-        <v>9680</v>
+        <v>9580</v>
       </c>
       <c r="E17" s="1">
-        <v>8906</v>
+        <v>8806</v>
       </c>
       <c r="F17" s="1">
-        <v>8134</v>
+        <v>8034</v>
       </c>
       <c r="G17" s="3">
         <v>7.1999999999999995E-2</v>
@@ -1256,7 +1256,7 @@
         <v>67</v>
       </c>
       <c r="B18" s="1">
-        <v>6344</v>
+        <v>6244</v>
       </c>
       <c r="C18" s="1">
         <v>4594</v>
@@ -1265,7 +1265,7 @@
         <v>4069</v>
       </c>
       <c r="E18" s="1">
-        <v>7339</v>
+        <v>7239</v>
       </c>
       <c r="F18" s="1">
         <v>3411</v>
@@ -1279,19 +1279,19 @@
         <v>68</v>
       </c>
       <c r="B19" s="1">
-        <v>10493</v>
+        <v>10393</v>
       </c>
       <c r="C19" s="1">
-        <v>7757</v>
+        <v>7657</v>
       </c>
       <c r="D19" s="1">
-        <v>6881</v>
+        <v>6781</v>
       </c>
       <c r="E19" s="1">
-        <v>6335</v>
+        <v>6235</v>
       </c>
       <c r="F19" s="1">
-        <v>5787</v>
+        <v>5687</v>
       </c>
       <c r="G19" s="3">
         <v>5.0999999999999997E-2</v>
@@ -1302,19 +1302,19 @@
         <v>69</v>
       </c>
       <c r="B20" s="1">
-        <v>26602</v>
+        <v>26502</v>
       </c>
       <c r="C20" s="1">
-        <v>19614</v>
+        <v>19514</v>
       </c>
       <c r="D20" s="1">
-        <v>17383</v>
+        <v>17283</v>
       </c>
       <c r="E20" s="1">
-        <v>15988</v>
+        <v>15888</v>
       </c>
       <c r="F20" s="1">
-        <v>14592</v>
+        <v>14492</v>
       </c>
       <c r="G20" s="3">
         <v>0.13</v>
@@ -1325,19 +1325,19 @@
         <v>71</v>
       </c>
       <c r="B21" s="1">
-        <v>24572</v>
+        <v>24472</v>
       </c>
       <c r="C21" s="1">
-        <v>18113</v>
+        <v>18013</v>
       </c>
       <c r="D21" s="1">
-        <v>16053</v>
+        <v>15953</v>
       </c>
       <c r="E21" s="1">
-        <v>14764</v>
+        <v>14664</v>
       </c>
       <c r="F21" s="1">
-        <v>13447</v>
+        <v>13347</v>
       </c>
       <c r="G21" s="3">
         <v>0.12</v>
@@ -1348,19 +1348,19 @@
         <v>72</v>
       </c>
       <c r="B22" s="1">
-        <v>24572</v>
+        <v>24472</v>
       </c>
       <c r="C22" s="1">
-        <v>18113</v>
+        <v>18013</v>
       </c>
       <c r="D22" s="1">
-        <v>16053</v>
+        <v>15953</v>
       </c>
       <c r="E22" s="1">
-        <v>14764</v>
+        <v>14664</v>
       </c>
       <c r="F22" s="1">
-        <v>13447</v>
+        <v>13347</v>
       </c>
       <c r="G22" s="3">
         <v>0.12</v>
@@ -1371,19 +1371,19 @@
         <v>77</v>
       </c>
       <c r="B23" s="1">
-        <v>26484</v>
+        <v>26384</v>
       </c>
       <c r="C23" s="1">
-        <v>15110</v>
+        <v>15010</v>
       </c>
       <c r="D23" s="1">
-        <v>13393</v>
+        <v>13293</v>
       </c>
       <c r="E23" s="1">
-        <v>12320</v>
+        <v>12220</v>
       </c>
       <c r="F23" s="1">
-        <v>11247</v>
+        <v>11147</v>
       </c>
       <c r="G23" s="3">
         <v>0.1</v>
@@ -1394,19 +1394,19 @@
         <v>187</v>
       </c>
       <c r="B24" s="1">
-        <v>27420</v>
+        <v>27320</v>
       </c>
       <c r="C24" s="1">
-        <v>20209</v>
+        <v>20109</v>
       </c>
       <c r="D24" s="1">
-        <v>17908</v>
+        <v>17808</v>
       </c>
       <c r="E24" s="1">
-        <v>16471</v>
+        <v>16371</v>
       </c>
       <c r="F24" s="1">
-        <v>15034</v>
+        <v>14934</v>
       </c>
       <c r="G24" s="3">
         <v>0.13400000000000001</v>
@@ -1417,19 +1417,19 @@
         <v>188</v>
       </c>
       <c r="B25" s="1">
-        <v>12738</v>
+        <v>12638</v>
       </c>
       <c r="C25" s="1">
-        <v>9407</v>
+        <v>9307</v>
       </c>
       <c r="D25" s="1">
-        <v>8344</v>
+        <v>8244</v>
       </c>
       <c r="E25" s="1">
-        <v>7679</v>
+        <v>7579</v>
       </c>
       <c r="F25" s="1">
-        <v>7013</v>
+        <v>6913</v>
       </c>
       <c r="G25" s="3">
         <v>6.2E-2</v>
@@ -1440,19 +1440,19 @@
         <v>896</v>
       </c>
       <c r="B26" s="1">
-        <v>29880</v>
+        <v>29780</v>
       </c>
       <c r="C26" s="1">
-        <v>22016</v>
+        <v>21916</v>
       </c>
       <c r="D26" s="1">
-        <v>19509</v>
+        <v>19409</v>
       </c>
       <c r="E26" s="1">
-        <v>17942</v>
+        <v>17842</v>
       </c>
       <c r="F26" s="1">
-        <v>16375</v>
+        <v>16275</v>
       </c>
       <c r="G26" s="3">
         <v>0.14599999999999999</v>
@@ -1463,19 +1463,19 @@
         <v>200</v>
       </c>
       <c r="B27" s="1">
-        <v>14381</v>
+        <v>14281</v>
       </c>
       <c r="C27" s="1">
-        <v>10612</v>
+        <v>10512</v>
       </c>
       <c r="D27" s="1">
-        <v>9410</v>
+        <v>9310</v>
       </c>
       <c r="E27" s="1">
-        <v>8659</v>
+        <v>8559</v>
       </c>
       <c r="F27" s="1">
-        <v>7907</v>
+        <v>7807</v>
       </c>
       <c r="G27" s="3">
         <v>7.0000000000000007E-2</v>
@@ -1486,19 +1486,19 @@
         <v>205</v>
       </c>
       <c r="B28" s="1">
-        <v>19057</v>
+        <v>18957</v>
       </c>
       <c r="C28" s="1">
-        <v>14053</v>
+        <v>13953</v>
       </c>
       <c r="D28" s="1">
-        <v>12456</v>
+        <v>12356</v>
       </c>
       <c r="E28" s="1">
-        <v>11459</v>
+        <v>11359</v>
       </c>
       <c r="F28" s="1">
-        <v>10460</v>
+        <v>10360</v>
       </c>
       <c r="G28" s="3">
         <v>9.2999999999999999E-2</v>
@@ -1509,19 +1509,19 @@
         <v>206</v>
       </c>
       <c r="B29" s="1">
-        <v>20075</v>
+        <v>19975</v>
       </c>
       <c r="C29" s="1">
-        <v>14797</v>
+        <v>14697</v>
       </c>
       <c r="D29" s="1">
-        <v>13115</v>
+        <v>13015</v>
       </c>
       <c r="E29" s="1">
-        <v>12063</v>
+        <v>11963</v>
       </c>
       <c r="F29" s="1">
-        <v>11011</v>
+        <v>10911</v>
       </c>
       <c r="G29" s="3">
         <v>9.8000000000000004E-2</v>
@@ -1532,19 +1532,19 @@
         <v>207</v>
       </c>
       <c r="B30" s="1">
-        <v>14381</v>
+        <v>14281</v>
       </c>
       <c r="C30" s="1">
-        <v>10612</v>
+        <v>10512</v>
       </c>
       <c r="D30" s="1">
-        <v>9410</v>
+        <v>9310</v>
       </c>
       <c r="E30" s="1">
-        <v>8659</v>
+        <v>8559</v>
       </c>
       <c r="F30" s="1">
-        <v>7907</v>
+        <v>7807</v>
       </c>
       <c r="G30" s="3">
         <v>7.0000000000000007E-2</v>
@@ -1555,19 +1555,19 @@
         <v>215</v>
       </c>
       <c r="B31" s="1">
-        <v>21912</v>
+        <v>21812</v>
       </c>
       <c r="C31" s="1">
-        <v>16158</v>
+        <v>16058</v>
       </c>
       <c r="D31" s="1">
-        <v>14320</v>
+        <v>14220</v>
       </c>
       <c r="E31" s="1">
-        <v>13171</v>
+        <v>13071</v>
       </c>
       <c r="F31" s="1">
-        <v>12023</v>
+        <v>11923</v>
       </c>
       <c r="G31" s="3">
         <v>0.107</v>
@@ -1578,19 +1578,19 @@
         <v>238</v>
       </c>
       <c r="B32" s="1">
-        <v>12438</v>
+        <v>12338</v>
       </c>
       <c r="C32" s="1">
-        <v>9707</v>
+        <v>9607</v>
       </c>
       <c r="D32" s="1">
-        <v>8344</v>
+        <v>8244</v>
       </c>
       <c r="E32" s="1">
-        <v>7679</v>
+        <v>7579</v>
       </c>
       <c r="F32" s="1">
-        <v>7013</v>
+        <v>6913</v>
       </c>
       <c r="G32" s="3">
         <v>6.2E-2</v>
@@ -1601,19 +1601,19 @@
         <v>264</v>
       </c>
       <c r="B33" s="1">
-        <v>27828</v>
+        <v>27728</v>
       </c>
       <c r="C33" s="1">
-        <v>20514</v>
+        <v>20414</v>
       </c>
       <c r="D33" s="1">
-        <v>18180</v>
+        <v>18080</v>
       </c>
       <c r="E33" s="1">
-        <v>16720</v>
+        <v>16620</v>
       </c>
       <c r="F33" s="1">
-        <v>15260</v>
+        <v>15160</v>
       </c>
       <c r="G33" s="3">
         <v>0.13600000000000001</v>
@@ -1624,7 +1624,7 @@
         <v>284</v>
       </c>
       <c r="B34" s="1">
-        <v>6166</v>
+        <v>6066</v>
       </c>
       <c r="C34" s="1">
         <v>4468</v>
@@ -1647,19 +1647,19 @@
         <v>289</v>
       </c>
       <c r="B35" s="1">
-        <v>34147</v>
+        <v>34047</v>
       </c>
       <c r="C35" s="1">
-        <v>25160</v>
+        <v>25060</v>
       </c>
       <c r="D35" s="1">
-        <v>22292</v>
+        <v>22192</v>
       </c>
       <c r="E35" s="1">
-        <v>20500</v>
+        <v>20400</v>
       </c>
       <c r="F35" s="1">
-        <v>18707</v>
+        <v>18607</v>
       </c>
       <c r="G35" s="3">
         <v>0.16700000000000001</v>
@@ -1670,19 +1670,19 @@
         <v>311</v>
       </c>
       <c r="B36" s="1">
-        <v>27112</v>
+        <v>27012</v>
       </c>
       <c r="C36" s="1">
-        <v>20061</v>
+        <v>19961</v>
       </c>
       <c r="D36" s="1">
-        <v>14777</v>
+        <v>14677</v>
       </c>
       <c r="E36" s="1">
-        <v>16350</v>
+        <v>16250</v>
       </c>
       <c r="F36" s="1">
-        <v>14992</v>
+        <v>14892</v>
       </c>
       <c r="G36" s="3">
         <v>0.13300000000000001</v>
@@ -1693,19 +1693,19 @@
         <v>312</v>
       </c>
       <c r="B37" s="1">
-        <v>27212</v>
+        <v>27112</v>
       </c>
       <c r="C37" s="1">
-        <v>20061</v>
+        <v>19961</v>
       </c>
       <c r="D37" s="1">
-        <v>14777</v>
+        <v>14677</v>
       </c>
       <c r="E37" s="1">
-        <v>16350</v>
+        <v>16250</v>
       </c>
       <c r="F37" s="1">
-        <v>14992</v>
+        <v>14892</v>
       </c>
       <c r="G37" s="3">
         <v>0.13300000000000001</v>
@@ -1725,7 +1725,7 @@
         <v>2259</v>
       </c>
       <c r="E38" s="1">
-        <v>8078</v>
+        <v>7978</v>
       </c>
       <c r="F38" s="1">
         <v>1895</v>
@@ -1739,19 +1739,19 @@
         <v>354</v>
       </c>
       <c r="B39" s="1">
-        <v>12329</v>
+        <v>12229</v>
       </c>
       <c r="C39" s="1">
-        <v>9103</v>
+        <v>9003</v>
       </c>
       <c r="D39" s="1">
-        <v>8073</v>
+        <v>7973</v>
       </c>
       <c r="E39" s="1">
-        <v>7429</v>
+        <v>7329</v>
       </c>
       <c r="F39" s="1">
-        <v>6784</v>
+        <v>6684</v>
       </c>
       <c r="G39" s="3">
         <v>0.06</v>
@@ -1762,19 +1762,19 @@
         <v>355</v>
       </c>
       <c r="B40" s="1">
-        <v>19057</v>
+        <v>18957</v>
       </c>
       <c r="C40" s="1">
-        <v>14053</v>
+        <v>13953</v>
       </c>
       <c r="D40" s="1">
-        <v>12456</v>
+        <v>12356</v>
       </c>
       <c r="E40" s="1">
-        <v>11459</v>
+        <v>11359</v>
       </c>
       <c r="F40" s="1">
-        <v>10960</v>
+        <v>10860</v>
       </c>
       <c r="G40" s="3">
         <v>9.2999999999999999E-2</v>
@@ -1785,19 +1785,19 @@
         <v>374</v>
       </c>
       <c r="B41" s="1">
-        <v>24512</v>
+        <v>24412</v>
       </c>
       <c r="C41" s="1">
-        <v>18113</v>
+        <v>18013</v>
       </c>
       <c r="D41" s="1">
-        <v>16053</v>
+        <v>15953</v>
       </c>
       <c r="E41" s="1">
-        <v>14764</v>
+        <v>14664</v>
       </c>
       <c r="F41" s="1">
-        <v>13447</v>
+        <v>13347</v>
       </c>
       <c r="G41" s="3">
         <v>0.12</v>
@@ -1808,19 +1808,19 @@
         <v>375</v>
       </c>
       <c r="B42" s="1">
-        <v>25993</v>
+        <v>25893</v>
       </c>
       <c r="C42" s="1">
-        <v>19168</v>
+        <v>19068</v>
       </c>
       <c r="D42" s="1">
-        <v>16987</v>
+        <v>16887</v>
       </c>
       <c r="E42" s="1">
-        <v>16562</v>
+        <v>16462</v>
       </c>
       <c r="F42" s="1">
-        <v>14261</v>
+        <v>14161</v>
       </c>
       <c r="G42" s="3">
         <v>0.127</v>
@@ -1831,19 +1831,19 @@
         <v>376</v>
       </c>
       <c r="B43" s="1">
-        <v>24572</v>
+        <v>24472</v>
       </c>
       <c r="C43" s="1">
-        <v>18113</v>
+        <v>18013</v>
       </c>
       <c r="D43" s="1">
-        <v>16053</v>
+        <v>15953</v>
       </c>
       <c r="E43" s="1">
-        <v>14764</v>
+        <v>14664</v>
       </c>
       <c r="F43" s="1">
-        <v>13447</v>
+        <v>13347</v>
       </c>
       <c r="G43" s="3">
         <v>0.12</v>
@@ -1854,19 +1854,19 @@
         <v>439</v>
       </c>
       <c r="B44" s="1">
-        <v>16411</v>
+        <v>16311</v>
       </c>
       <c r="C44" s="1">
-        <v>12106</v>
+        <v>12006</v>
       </c>
       <c r="D44" s="1">
-        <v>10732</v>
+        <v>10632</v>
       </c>
       <c r="E44" s="1">
-        <v>9873</v>
+        <v>9773</v>
       </c>
       <c r="F44" s="1">
-        <v>9015</v>
+        <v>8915</v>
       </c>
       <c r="G44" s="3">
         <v>0.08</v>
@@ -1877,19 +1877,19 @@
         <v>456</v>
       </c>
       <c r="B45" s="1">
-        <v>210303</v>
+        <v>209803</v>
       </c>
       <c r="C45" s="1">
-        <v>154934</v>
+        <v>154434</v>
       </c>
       <c r="D45" s="1">
-        <v>137266</v>
+        <v>136766</v>
       </c>
       <c r="E45" s="1">
-        <v>126224</v>
+        <v>125724</v>
       </c>
       <c r="F45" s="1">
-        <v>115181</v>
+        <v>114681</v>
       </c>
       <c r="G45" s="3">
         <v>1.0289999999999999</v>
@@ -1900,19 +1900,19 @@
         <v>457</v>
       </c>
       <c r="B46" s="1">
-        <v>210303</v>
+        <v>209803</v>
       </c>
       <c r="C46" s="1">
-        <v>154934</v>
+        <v>154434</v>
       </c>
       <c r="D46" s="1">
-        <v>137266</v>
+        <v>136766</v>
       </c>
       <c r="E46" s="1">
-        <v>126224</v>
+        <v>125724</v>
       </c>
       <c r="F46" s="1">
-        <v>115181</v>
+        <v>114681</v>
       </c>
       <c r="G46" s="3">
         <v>1.0289999999999999</v>
@@ -1923,19 +1923,19 @@
         <v>463</v>
       </c>
       <c r="B47" s="1">
-        <v>23346</v>
+        <v>23246</v>
       </c>
       <c r="C47" s="1">
-        <v>17213</v>
+        <v>17113</v>
       </c>
       <c r="D47" s="1">
-        <v>15256</v>
+        <v>15156</v>
       </c>
       <c r="E47" s="1">
-        <v>14031</v>
+        <v>13931</v>
       </c>
       <c r="F47" s="1">
-        <v>12808</v>
+        <v>12708</v>
       </c>
       <c r="G47" s="3">
         <v>0.114</v>
@@ -1946,19 +1946,19 @@
         <v>471</v>
       </c>
       <c r="B48" s="1">
-        <v>24967</v>
+        <v>24867</v>
       </c>
       <c r="C48" s="1">
-        <v>18417</v>
+        <v>18317</v>
       </c>
       <c r="D48" s="1">
-        <v>16323</v>
+        <v>16223</v>
       </c>
       <c r="E48" s="1">
-        <v>15012</v>
+        <v>14912</v>
       </c>
       <c r="F48" s="1">
-        <v>13702</v>
+        <v>13602</v>
       </c>
       <c r="G48" s="3">
         <v>0.12</v>
@@ -1969,19 +1969,19 @@
         <v>504</v>
       </c>
       <c r="B49" s="1">
-        <v>61795</v>
+        <v>61695</v>
       </c>
       <c r="C49" s="1">
-        <v>45573</v>
+        <v>45473</v>
       </c>
       <c r="D49" s="1">
-        <v>40349</v>
+        <v>40249</v>
       </c>
       <c r="E49" s="1">
-        <v>37132</v>
+        <v>37032</v>
       </c>
       <c r="F49" s="1">
-        <v>33885</v>
+        <v>33785</v>
       </c>
       <c r="G49" s="3">
         <v>0.3</v>
@@ -1992,7 +1992,7 @@
         <v>520</v>
       </c>
       <c r="B50" s="1">
-        <v>42667</v>
+        <v>42567</v>
       </c>
       <c r="C50" s="1">
         <v>3152</v>
@@ -2001,7 +2001,7 @@
         <v>2393</v>
       </c>
       <c r="E50" s="1">
-        <v>9568</v>
+        <v>9468</v>
       </c>
       <c r="F50" s="1">
         <v>2345</v>
@@ -2015,19 +2015,19 @@
         <v>523</v>
       </c>
       <c r="B51" s="1">
-        <v>19730</v>
+        <v>19630</v>
       </c>
       <c r="C51" s="1">
-        <v>9400</v>
+        <v>9300</v>
       </c>
       <c r="D51" s="1">
-        <v>8337</v>
+        <v>8237</v>
       </c>
       <c r="E51" s="1">
-        <v>76672</v>
+        <v>76572</v>
       </c>
       <c r="F51" s="1">
-        <v>7008</v>
+        <v>6908</v>
       </c>
       <c r="G51" s="3">
         <v>0.06</v>
@@ -2038,19 +2038,19 @@
         <v>528</v>
       </c>
       <c r="B52" s="1">
-        <v>119980</v>
+        <v>119480</v>
       </c>
       <c r="C52" s="1">
-        <v>88051</v>
+        <v>87951</v>
       </c>
       <c r="D52" s="1">
-        <v>77990</v>
+        <v>77890</v>
       </c>
       <c r="E52" s="1">
-        <v>71703</v>
+        <v>71603</v>
       </c>
       <c r="F52" s="1">
-        <v>65414</v>
+        <v>65314</v>
       </c>
       <c r="G52" s="3">
         <v>0.57999999999999996</v>
@@ -2061,19 +2061,19 @@
         <v>529</v>
       </c>
       <c r="B53" s="1">
-        <v>119980</v>
+        <v>119480</v>
       </c>
       <c r="C53" s="1">
-        <v>88051</v>
+        <v>87951</v>
       </c>
       <c r="D53" s="1">
-        <v>77990</v>
+        <v>77890</v>
       </c>
       <c r="E53" s="1">
-        <v>71703</v>
+        <v>71603</v>
       </c>
       <c r="F53" s="1">
-        <v>65414</v>
+        <v>65314</v>
       </c>
       <c r="G53" s="3">
         <v>0.57999999999999996</v>
@@ -2084,19 +2084,19 @@
         <v>532</v>
       </c>
       <c r="B54" s="1">
-        <v>119980</v>
+        <v>119480</v>
       </c>
       <c r="C54" s="1">
-        <v>88051</v>
+        <v>87951</v>
       </c>
       <c r="D54" s="1">
-        <v>77990</v>
+        <v>77890</v>
       </c>
       <c r="E54" s="1">
-        <v>71703</v>
+        <v>71603</v>
       </c>
       <c r="F54" s="1">
-        <v>65414</v>
+        <v>65314</v>
       </c>
       <c r="G54" s="3">
         <v>0.57999999999999996</v>
@@ -2107,19 +2107,19 @@
         <v>536</v>
       </c>
       <c r="B55" s="1">
-        <v>119980</v>
+        <v>119480</v>
       </c>
       <c r="C55" s="1">
-        <v>88051</v>
+        <v>87951</v>
       </c>
       <c r="D55" s="1">
-        <v>77990</v>
+        <v>77890</v>
       </c>
       <c r="E55" s="1">
-        <v>71703</v>
+        <v>71603</v>
       </c>
       <c r="F55" s="1">
-        <v>65414</v>
+        <v>65314</v>
       </c>
       <c r="G55" s="3">
         <v>0.57999999999999996</v>
@@ -2130,19 +2130,19 @@
         <v>547</v>
       </c>
       <c r="B56" s="1">
-        <v>98385</v>
+        <v>98285</v>
       </c>
       <c r="C56" s="1">
-        <v>72448</v>
+        <v>72348</v>
       </c>
       <c r="D56" s="1">
-        <v>64172</v>
+        <v>64072</v>
       </c>
       <c r="E56" s="1">
-        <v>59000</v>
+        <v>58900</v>
       </c>
       <c r="F56" s="1">
-        <v>53826</v>
+        <v>53726</v>
       </c>
       <c r="G56" s="3">
         <v>0.48</v>
@@ -2153,19 +2153,19 @@
         <v>548</v>
       </c>
       <c r="B57" s="1">
-        <v>98385</v>
+        <v>98285</v>
       </c>
       <c r="C57" s="1">
-        <v>72448</v>
+        <v>72348</v>
       </c>
       <c r="D57" s="1">
-        <v>64172</v>
+        <v>64072</v>
       </c>
       <c r="E57" s="1">
-        <v>59000</v>
+        <v>58900</v>
       </c>
       <c r="F57" s="1">
-        <v>53826</v>
+        <v>53726</v>
       </c>
       <c r="G57" s="3">
         <v>0.48</v>
@@ -2176,19 +2176,19 @@
         <v>551</v>
       </c>
       <c r="B58" s="1">
-        <v>50979</v>
+        <v>50879</v>
       </c>
       <c r="C58" s="1">
-        <v>37589</v>
+        <v>37489</v>
       </c>
       <c r="D58" s="1">
-        <v>33305</v>
+        <v>33205</v>
       </c>
       <c r="E58" s="1">
-        <v>30627</v>
+        <v>30527</v>
       </c>
       <c r="F58" s="1">
-        <v>27949</v>
+        <v>27849</v>
       </c>
       <c r="G58" s="3">
         <v>0.2</v>
@@ -2199,19 +2199,19 @@
         <v>554</v>
       </c>
       <c r="B59" s="1">
-        <v>22967</v>
+        <v>22867</v>
       </c>
       <c r="C59" s="1">
-        <v>16953</v>
+        <v>16853</v>
       </c>
       <c r="D59" s="1">
-        <v>15027</v>
+        <v>14927</v>
       </c>
       <c r="E59" s="1">
-        <v>13824</v>
+        <v>13724</v>
       </c>
       <c r="F59" s="1">
-        <v>12679</v>
+        <v>12579</v>
       </c>
       <c r="G59" s="3">
         <v>0.11</v>
@@ -2222,16 +2222,16 @@
         <v>555</v>
       </c>
       <c r="B60" s="1">
-        <v>36549</v>
+        <v>36449</v>
       </c>
       <c r="C60" s="1">
-        <v>26959</v>
+        <v>26859</v>
       </c>
       <c r="D60" s="1">
-        <v>23889</v>
+        <v>23789</v>
       </c>
       <c r="E60" s="1">
-        <v>21970</v>
+        <v>21870</v>
       </c>
       <c r="F60" s="1">
         <v>2052</v>
@@ -2245,19 +2245,19 @@
         <v>556</v>
       </c>
       <c r="B61" s="1">
-        <v>36474</v>
+        <v>36374</v>
       </c>
       <c r="C61" s="1">
-        <v>26907</v>
+        <v>26807</v>
       </c>
       <c r="D61" s="1">
-        <v>23845</v>
+        <v>23745</v>
       </c>
       <c r="E61" s="1">
-        <v>21932</v>
+        <v>21832</v>
       </c>
       <c r="F61" s="1">
-        <v>20017</v>
+        <v>19917</v>
       </c>
       <c r="G61" s="3">
         <v>0.17</v>
@@ -2268,19 +2268,19 @@
         <v>558</v>
       </c>
       <c r="B62" s="1">
-        <v>40794</v>
+        <v>40694</v>
       </c>
       <c r="C62" s="1">
-        <v>30089</v>
+        <v>29989</v>
       </c>
       <c r="D62" s="1">
-        <v>26662</v>
+        <v>26562</v>
       </c>
       <c r="E62" s="1">
-        <v>24520</v>
+        <v>24420</v>
       </c>
       <c r="F62" s="1">
-        <v>22374</v>
+        <v>22274</v>
       </c>
       <c r="G62" s="3">
         <v>0.2</v>
@@ -2291,19 +2291,19 @@
         <v>559</v>
       </c>
       <c r="B63" s="1">
-        <v>14968</v>
+        <v>14868</v>
       </c>
       <c r="C63" s="1">
-        <v>11050</v>
+        <v>10950</v>
       </c>
       <c r="D63" s="1">
         <v>3798</v>
       </c>
       <c r="E63" s="1">
-        <v>9615</v>
+        <v>9515</v>
       </c>
       <c r="F63" s="1">
-        <v>8230</v>
+        <v>8130</v>
       </c>
       <c r="G63" s="3">
         <v>7.0000000000000007E-2</v>
@@ -2314,19 +2314,19 @@
         <v>560</v>
       </c>
       <c r="B64" s="1">
-        <v>17830</v>
+        <v>17730</v>
       </c>
       <c r="C64" s="1">
-        <v>13162</v>
+        <v>13062</v>
       </c>
       <c r="D64" s="1">
-        <v>11669</v>
+        <v>11569</v>
       </c>
       <c r="E64" s="1">
-        <v>10735</v>
+        <v>10635</v>
       </c>
       <c r="F64" s="1">
-        <v>9803</v>
+        <v>9703</v>
       </c>
       <c r="G64" s="3">
         <v>0.08</v>
@@ -2337,19 +2337,19 @@
         <v>561</v>
       </c>
       <c r="B65" s="1">
-        <v>14968</v>
+        <v>14868</v>
       </c>
       <c r="C65" s="1">
-        <v>11050</v>
+        <v>10950</v>
       </c>
       <c r="D65" s="1">
-        <v>9798</v>
+        <v>9698</v>
       </c>
       <c r="E65" s="1">
-        <v>9015</v>
+        <v>8915</v>
       </c>
       <c r="F65" s="1">
-        <v>8230</v>
+        <v>8130</v>
       </c>
       <c r="G65" s="3">
         <v>7.0000000000000007E-2</v>
@@ -2360,19 +2360,19 @@
         <v>563</v>
       </c>
       <c r="B66" s="1">
-        <v>23346</v>
+        <v>23246</v>
       </c>
       <c r="C66" s="1">
-        <v>17213</v>
+        <v>17113</v>
       </c>
       <c r="D66" s="1">
-        <v>15256</v>
+        <v>15156</v>
       </c>
       <c r="E66" s="1">
-        <v>14031</v>
+        <v>13931</v>
       </c>
       <c r="F66" s="1">
-        <v>12808</v>
+        <v>12708</v>
       </c>
       <c r="G66" s="3">
         <v>0.114</v>
@@ -2383,19 +2383,19 @@
         <v>564</v>
       </c>
       <c r="B67" s="1">
-        <v>12329</v>
+        <v>12229</v>
       </c>
       <c r="C67" s="1">
-        <v>9103</v>
+        <v>9003</v>
       </c>
       <c r="D67" s="1">
-        <v>8073</v>
+        <v>7973</v>
       </c>
       <c r="E67" s="1">
-        <v>7430</v>
+        <v>7330</v>
       </c>
       <c r="F67" s="1">
-        <v>6786</v>
+        <v>6686</v>
       </c>
       <c r="G67" s="3">
         <v>0.06</v>
@@ -2406,19 +2406,19 @@
         <v>566</v>
       </c>
       <c r="B68" s="1">
-        <v>30244</v>
+        <v>30144</v>
       </c>
       <c r="C68" s="1">
-        <v>22313</v>
+        <v>22213</v>
       </c>
       <c r="D68" s="1">
-        <v>19774</v>
+        <v>19674</v>
       </c>
       <c r="E68" s="1">
-        <v>18188</v>
+        <v>18088</v>
       </c>
       <c r="F68" s="1">
-        <v>16602</v>
+        <v>16502</v>
       </c>
       <c r="G68" s="3">
         <v>0.14000000000000001</v>
@@ -2429,19 +2429,19 @@
         <v>610</v>
       </c>
       <c r="B69" s="1">
-        <v>30074</v>
+        <v>29974</v>
       </c>
       <c r="C69" s="1">
-        <v>22173</v>
+        <v>22073</v>
       </c>
       <c r="D69" s="1">
-        <v>19648</v>
+        <v>19548</v>
       </c>
       <c r="E69" s="1">
-        <v>18071</v>
+        <v>17971</v>
       </c>
       <c r="F69" s="1">
-        <v>16492</v>
+        <v>16392</v>
       </c>
       <c r="G69" s="3">
         <v>0.14000000000000001</v>
@@ -2452,19 +2452,19 @@
         <v>612</v>
       </c>
       <c r="B70" s="1">
-        <v>13154</v>
+        <v>13054</v>
       </c>
       <c r="C70" s="1">
-        <v>9704</v>
+        <v>9604</v>
       </c>
       <c r="D70" s="1">
-        <v>8605</v>
+        <v>8505</v>
       </c>
       <c r="E70" s="1">
-        <v>7918</v>
+        <v>7818</v>
       </c>
       <c r="F70" s="1">
-        <v>7231</v>
+        <v>7131</v>
       </c>
       <c r="G70" s="3">
         <v>0.06</v>
@@ -2475,19 +2475,19 @@
         <v>613</v>
       </c>
       <c r="B71" s="1">
-        <v>65631</v>
+        <v>65531</v>
       </c>
       <c r="C71" s="1">
-        <v>48384</v>
+        <v>48284</v>
       </c>
       <c r="D71" s="1">
-        <v>42865</v>
+        <v>42765</v>
       </c>
       <c r="E71" s="1">
-        <v>39416</v>
+        <v>39316</v>
       </c>
       <c r="F71" s="1">
-        <v>35968</v>
+        <v>35868</v>
       </c>
       <c r="G71" s="3">
         <v>7.2999999999999995E-2</v>
@@ -2498,19 +2498,19 @@
         <v>618</v>
       </c>
       <c r="B72" s="1">
-        <v>28646</v>
+        <v>28546</v>
       </c>
       <c r="C72" s="1">
-        <v>21116</v>
+        <v>21016</v>
       </c>
       <c r="D72" s="1">
-        <v>18712</v>
+        <v>18612</v>
       </c>
       <c r="E72" s="1">
-        <v>17210</v>
+        <v>17110</v>
       </c>
       <c r="F72" s="1">
-        <v>15704</v>
+        <v>15604</v>
       </c>
       <c r="G72" s="3">
         <v>0.1</v>
@@ -2521,19 +2521,19 @@
         <v>621</v>
       </c>
       <c r="B73" s="1">
-        <v>31509</v>
+        <v>31409</v>
       </c>
       <c r="C73" s="1">
-        <v>93213</v>
+        <v>93113</v>
       </c>
       <c r="D73" s="1">
-        <v>20569</v>
+        <v>20469</v>
       </c>
       <c r="E73" s="1">
-        <v>18915</v>
+        <v>18815</v>
       </c>
       <c r="F73" s="1">
-        <v>17262</v>
+        <v>17162</v>
       </c>
       <c r="G73" s="3">
         <v>0.15</v>
@@ -2544,19 +2544,19 @@
         <v>622</v>
       </c>
       <c r="B74" s="1">
-        <v>68196</v>
+        <v>68096</v>
       </c>
       <c r="C74" s="1">
-        <v>50235</v>
+        <v>50135</v>
       </c>
       <c r="D74" s="1">
-        <v>44500</v>
+        <v>44400</v>
       </c>
       <c r="E74" s="1">
-        <v>40917</v>
+        <v>40817</v>
       </c>
       <c r="F74" s="1">
-        <v>37333</v>
+        <v>37233</v>
       </c>
       <c r="G74" s="3">
         <v>0.33</v>
@@ -2567,19 +2567,19 @@
         <v>624</v>
       </c>
       <c r="B75" s="1">
-        <v>28646</v>
+        <v>28546</v>
       </c>
       <c r="C75" s="1">
-        <v>21116</v>
+        <v>21016</v>
       </c>
       <c r="D75" s="1">
-        <v>18712</v>
+        <v>18612</v>
       </c>
       <c r="E75" s="1">
-        <v>17210</v>
+        <v>17110</v>
       </c>
       <c r="F75" s="1">
-        <v>15704</v>
+        <v>15604</v>
       </c>
       <c r="G75" s="3">
         <v>0.1</v>
@@ -2590,19 +2590,19 @@
         <v>633</v>
       </c>
       <c r="B76" s="1">
-        <v>15384</v>
+        <v>15284</v>
       </c>
       <c r="C76" s="1">
-        <v>11355</v>
+        <v>11255</v>
       </c>
       <c r="D76" s="1">
-        <v>10068</v>
+        <v>9968</v>
       </c>
       <c r="E76" s="1">
-        <v>9263</v>
+        <v>9163</v>
       </c>
       <c r="F76" s="1">
-        <v>8459</v>
+        <v>8359</v>
       </c>
       <c r="G76" s="3">
         <v>7.0000000000000007E-2</v>
@@ -2613,7 +2613,7 @@
         <v>634</v>
       </c>
       <c r="B77" s="1">
-        <v>306163</v>
+        <v>305663</v>
       </c>
       <c r="C77" s="1"/>
       <c r="D77" s="1"/>
@@ -2628,7 +2628,7 @@
         <v>635</v>
       </c>
       <c r="B78" s="1">
-        <v>306885</v>
+        <v>306385</v>
       </c>
       <c r="C78" s="1"/>
       <c r="D78" s="1"/>
@@ -2643,19 +2643,19 @@
         <v>640</v>
       </c>
       <c r="B79" s="1">
-        <v>17830</v>
+        <v>17730</v>
       </c>
       <c r="C79" s="1">
-        <v>13162</v>
+        <v>13062</v>
       </c>
       <c r="D79" s="1">
-        <v>11669</v>
+        <v>11569</v>
       </c>
       <c r="E79" s="1">
-        <v>10735</v>
+        <v>10635</v>
       </c>
       <c r="F79" s="1">
-        <v>9803</v>
+        <v>9703</v>
       </c>
       <c r="G79" s="3">
         <v>0.08</v>
@@ -2666,19 +2666,19 @@
         <v>641</v>
       </c>
       <c r="B80" s="1">
-        <v>19027</v>
+        <v>18927</v>
       </c>
       <c r="C80" s="1">
-        <v>14053</v>
+        <v>13953</v>
       </c>
       <c r="D80" s="1">
-        <v>12460</v>
+        <v>12360</v>
       </c>
       <c r="E80" s="1">
-        <v>11463</v>
+        <v>11363</v>
       </c>
       <c r="F80" s="1">
-        <v>10467</v>
+        <v>10367</v>
       </c>
       <c r="G80" s="3">
         <v>0.09</v>
@@ -2689,19 +2689,19 @@
         <v>642</v>
       </c>
       <c r="B81" s="1">
-        <v>22707</v>
+        <v>22607</v>
       </c>
       <c r="C81" s="1">
-        <v>16759</v>
+        <v>16659</v>
       </c>
       <c r="D81" s="1">
-        <v>14857</v>
+        <v>14757</v>
       </c>
       <c r="E81" s="1">
-        <v>13666</v>
+        <v>13566</v>
       </c>
       <c r="F81" s="1">
-        <v>72496</v>
+        <v>72396</v>
       </c>
       <c r="G81" s="3">
         <v>0.11</v>
@@ -2712,19 +2712,19 @@
         <v>643</v>
       </c>
       <c r="B82" s="1">
-        <v>27398</v>
+        <v>27298</v>
       </c>
       <c r="C82" s="1">
-        <v>20209</v>
+        <v>20109</v>
       </c>
       <c r="D82" s="1">
-        <v>17911</v>
+        <v>17811</v>
       </c>
       <c r="E82" s="1">
-        <v>16474</v>
+        <v>16374</v>
       </c>
       <c r="F82" s="1">
-        <v>15037</v>
+        <v>14937</v>
       </c>
       <c r="G82" s="3">
         <v>0.13</v>
@@ -2735,19 +2735,19 @@
         <v>644</v>
       </c>
       <c r="B83" s="1">
-        <v>27398</v>
+        <v>27298</v>
       </c>
       <c r="C83" s="1">
-        <v>20209</v>
+        <v>20109</v>
       </c>
       <c r="D83" s="1">
-        <v>17911</v>
+        <v>17811</v>
       </c>
       <c r="E83" s="1">
-        <v>16474</v>
+        <v>16374</v>
       </c>
       <c r="F83" s="1">
-        <v>15037</v>
+        <v>14937</v>
       </c>
       <c r="G83" s="3">
         <v>0.13</v>
@@ -2758,19 +2758,19 @@
         <v>645</v>
       </c>
       <c r="B84" s="1">
-        <v>29835</v>
+        <v>29735</v>
       </c>
       <c r="C84" s="1">
-        <v>22008</v>
+        <v>21908</v>
       </c>
       <c r="D84" s="1">
-        <v>19504</v>
+        <v>19404</v>
       </c>
       <c r="E84" s="1">
-        <v>17937</v>
+        <v>17837</v>
       </c>
       <c r="F84" s="1">
-        <v>16393</v>
+        <v>16293</v>
       </c>
       <c r="G84" s="3">
         <v>0.14000000000000001</v>
@@ -2781,19 +2781,19 @@
         <v>646</v>
       </c>
       <c r="B85" s="1">
-        <v>18432</v>
+        <v>18332</v>
       </c>
       <c r="C85" s="1">
-        <v>13607</v>
+        <v>13507</v>
       </c>
       <c r="D85" s="1">
-        <v>12064</v>
+        <v>11964</v>
       </c>
       <c r="E85" s="1">
-        <v>11100</v>
+        <v>11000</v>
       </c>
       <c r="F85" s="1">
-        <v>10135</v>
+        <v>10035</v>
       </c>
       <c r="G85" s="3">
         <v>0.09</v>
@@ -2804,19 +2804,19 @@
         <v>647</v>
       </c>
       <c r="B86" s="1">
-        <v>18648</v>
+        <v>18548</v>
       </c>
       <c r="C86" s="1">
-        <v>13764</v>
+        <v>13664</v>
       </c>
       <c r="D86" s="1">
-        <v>12202</v>
+        <v>12102</v>
       </c>
       <c r="E86" s="1">
-        <v>17226</v>
+        <v>17126</v>
       </c>
       <c r="F86" s="1">
-        <v>10250</v>
+        <v>10150</v>
       </c>
       <c r="G86" s="3">
         <v>0.09</v>
@@ -2827,19 +2827,19 @@
         <v>651</v>
       </c>
       <c r="B87" s="1">
-        <v>30244</v>
+        <v>30144</v>
       </c>
       <c r="C87" s="1">
-        <v>22313</v>
+        <v>22213</v>
       </c>
       <c r="D87" s="1">
-        <v>19774</v>
+        <v>19674</v>
       </c>
       <c r="E87" s="1">
-        <v>18188</v>
+        <v>18088</v>
       </c>
       <c r="F87" s="1">
-        <v>16602</v>
+        <v>16502</v>
       </c>
       <c r="G87" s="3">
         <v>0.14000000000000001</v>
@@ -2850,19 +2850,19 @@
         <v>653</v>
       </c>
       <c r="B88" s="1">
-        <v>24744</v>
+        <v>24644</v>
       </c>
       <c r="C88" s="1">
-        <v>18261</v>
+        <v>18161</v>
       </c>
       <c r="D88" s="1">
-        <v>16186</v>
+        <v>16086</v>
       </c>
       <c r="E88" s="1">
-        <v>14890</v>
+        <v>14790</v>
       </c>
       <c r="F88" s="1">
-        <v>73593</v>
+        <v>73493</v>
       </c>
       <c r="G88" s="3">
         <v>0.12</v>
@@ -2873,19 +2873,19 @@
         <v>654</v>
       </c>
       <c r="B89" s="1">
-        <v>28646</v>
+        <v>28546</v>
       </c>
       <c r="C89" s="1">
-        <v>221138</v>
+        <v>220638</v>
       </c>
       <c r="D89" s="1">
-        <v>18733</v>
+        <v>18633</v>
       </c>
       <c r="E89" s="1">
-        <v>17231</v>
+        <v>17131</v>
       </c>
       <c r="F89" s="1">
-        <v>15729</v>
+        <v>15629</v>
       </c>
       <c r="G89" s="3">
         <v>0.1</v>
@@ -2896,19 +2896,19 @@
         <v>656</v>
       </c>
       <c r="B90" s="1">
-        <v>45529</v>
+        <v>45429</v>
       </c>
       <c r="C90" s="1">
-        <v>33575</v>
+        <v>33475</v>
       </c>
       <c r="D90" s="1">
-        <v>29751</v>
+        <v>29651</v>
       </c>
       <c r="E90" s="1">
-        <v>27359</v>
+        <v>27259</v>
       </c>
       <c r="F90" s="1">
-        <v>24968</v>
+        <v>24868</v>
       </c>
       <c r="G90" s="3">
         <v>0.22</v>
@@ -2919,19 +2919,19 @@
         <v>659</v>
       </c>
       <c r="B91" s="1">
-        <v>109178</v>
+        <v>108678</v>
       </c>
       <c r="C91" s="1">
-        <v>86090</v>
+        <v>85990</v>
       </c>
       <c r="D91" s="1">
-        <v>40988</v>
+        <v>40888</v>
       </c>
       <c r="E91" s="1">
-        <v>65219</v>
+        <v>65119</v>
       </c>
       <c r="F91" s="1">
-        <v>59499</v>
+        <v>59399</v>
       </c>
       <c r="G91" s="3">
         <v>0.53</v>
@@ -2942,19 +2942,19 @@
         <v>664</v>
       </c>
       <c r="B92" s="1">
-        <v>25963</v>
+        <v>25863</v>
       </c>
       <c r="C92" s="1">
-        <v>19161</v>
+        <v>19061</v>
       </c>
       <c r="D92" s="1">
-        <v>16983</v>
+        <v>16883</v>
       </c>
       <c r="E92" s="1">
-        <v>15622</v>
+        <v>15522</v>
       </c>
       <c r="F92" s="1">
-        <v>17460</v>
+        <v>17360</v>
       </c>
       <c r="G92" s="3">
         <v>0.12</v>
@@ -2965,7 +2965,7 @@
         <v>716</v>
       </c>
       <c r="B93" s="1">
-        <v>6404</v>
+        <v>6304</v>
       </c>
       <c r="C93" s="1">
         <v>4646</v>

</xml_diff>